<commit_message>
Analysis List and Progress
</commit_message>
<xml_diff>
--- a/backend/POC/prefilter_cache.xlsx
+++ b/backend/POC/prefilter_cache.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="55">
   <si>
     <t>process_hash</t>
   </si>
@@ -43,9 +43,42 @@
     <t>Test_Merchant</t>
   </si>
   <si>
+    <t>Test3</t>
+  </si>
+  <si>
+    <t>d</t>
+  </si>
+  <si>
+    <t>eee</t>
+  </si>
+  <si>
+    <t>test</t>
+  </si>
+  <si>
+    <t>Custom_Regulation</t>
+  </si>
+  <si>
+    <t>tesr</t>
+  </si>
+  <si>
+    <t>e</t>
+  </si>
+  <si>
+    <t>t</t>
+  </si>
+  <si>
     <t>1</t>
   </si>
   <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
     <t>All payment service providers shall conduct a comprehensive identity verification of each merchant prior to granting access to payment processing services.</t>
   </si>
   <si>
@@ -101,6 +134,54 @@
   </si>
   <si>
     <t>Staff supporting merchant accounts must receive adequate and up-to-date compliance training that is sufficient to enable them to perform their duties competently.</t>
+  </si>
+  <si>
+    <t>All payment service providers shall conduct a comprehensive identity verification of each merchant prior to granting access to payment processing services.
+The identity verification process must incl</t>
+  </si>
+  <si>
+    <t>7	All payment service providers shall conduct a comprehensive identity verification of each merchant prior to granting access to payment processing services.
+8	The identity verification process must i</t>
+  </si>
+  <si>
+    <t>7	All payment service providers shall conduct a comprehensive identity verification of each merchant prior to granting access to payment processing services. its important for all payment processes. 8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7	All payment service providers shall conduct a comprehensive identity verification of each merchant prior to granting access to payment processing services. its important for all payment processes.
+</t>
+  </si>
+  <si>
+    <t>7 All payment service providers shall conduct a comprehensive identity verification of each merchant prior to granting access to payment processing services.</t>
+  </si>
+  <si>
+    <t>8 The identity verification process must include validation of the merchant's legal registration, beneficial ownership structure, and principal place of business.</t>
+  </si>
+  <si>
+    <t>9 Payment service providers are prohibited from onboarding any merchant that appears on a government-maintained sanctions or exclusion list.</t>
+  </si>
+  <si>
+    <t>10 Where a merchant operates in a high-risk category as defined in Annex II, the payment service provider shall apply enhanced due diligence measures appropriate to the level of risk.</t>
+  </si>
+  <si>
+    <t>11 Verification records shall be retained for a minimum period of seven years from the date of merchant account closure.</t>
+  </si>
+  <si>
+    <t>12 This chapter outlines the obligations of payment service providers with respect to consumer data collected during payment processing.</t>
+  </si>
+  <si>
+    <t>13 Payment service providers shall implement adequate technical and organizational safeguards to protect consumer data against unauthorized access, disclosure, or destruction.</t>
+  </si>
+  <si>
+    <t>7 All payment service providers shall conduct a comprehensive identity verification of each merchant prior to granting access to payment processing services. obligation</t>
+  </si>
+  <si>
+    <t>8 The identity verification process must include validation of the merchant's legal registration, beneficial ownership structure, and principal place of business. obligation</t>
+  </si>
+  <si>
+    <t>9 Payment service providers are prohibited from onboarding any merchant that appears on a government-maintained sanctions or exclusion list. prohibition</t>
+  </si>
+  <si>
+    <t>10 Where a merchant operates in a high-risk category as defined in Annex II, the payment service provider shall apply enhanced due diligence measures appropriate to the level of risk. obligation</t>
   </si>
 </sst>
 </file>
@@ -432,7 +513,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -466,7 +547,7 @@
         <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E2">
         <v>0.5838</v>
@@ -486,7 +567,7 @@
         <v>8</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="E3">
         <v>0.6263</v>
@@ -506,7 +587,7 @@
         <v>9</v>
       </c>
       <c r="D4" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E4">
         <v>0.6303</v>
@@ -526,7 +607,7 @@
         <v>10</v>
       </c>
       <c r="D5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="E5">
         <v>0.6439</v>
@@ -546,7 +627,7 @@
         <v>11</v>
       </c>
       <c r="D6" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="E6">
         <v>0.4402</v>
@@ -566,7 +647,7 @@
         <v>12</v>
       </c>
       <c r="D7" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="E7">
         <v>0.6491</v>
@@ -586,7 +667,7 @@
         <v>13</v>
       </c>
       <c r="D8" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="E8">
         <v>0.6712</v>
@@ -606,7 +687,7 @@
         <v>14</v>
       </c>
       <c r="D9" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="E9">
         <v>0.5116000000000001</v>
@@ -626,7 +707,7 @@
         <v>15</v>
       </c>
       <c r="D10" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="E10">
         <v>0.5103</v>
@@ -646,7 +727,7 @@
         <v>16</v>
       </c>
       <c r="D11" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="E11">
         <v>0.521</v>
@@ -666,7 +747,7 @@
         <v>17</v>
       </c>
       <c r="D12" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="E12">
         <v>0.7005</v>
@@ -686,7 +767,7 @@
         <v>18</v>
       </c>
       <c r="D13" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="E13">
         <v>0.4253</v>
@@ -706,7 +787,7 @@
         <v>19</v>
       </c>
       <c r="D14" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="E14">
         <v>0.4379</v>
@@ -726,7 +807,7 @@
         <v>20</v>
       </c>
       <c r="D15" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="E15">
         <v>0.6097</v>
@@ -746,7 +827,7 @@
         <v>21</v>
       </c>
       <c r="D16" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="E16">
         <v>0.4384</v>
@@ -766,7 +847,7 @@
         <v>22</v>
       </c>
       <c r="D17" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="E17">
         <v>0.427</v>
@@ -786,7 +867,7 @@
         <v>27</v>
       </c>
       <c r="D18" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="E18">
         <v>0.6855</v>
@@ -806,7 +887,7 @@
         <v>28</v>
       </c>
       <c r="D19" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="E19">
         <v>0.5853</v>
@@ -826,7 +907,7 @@
         <v>29</v>
       </c>
       <c r="D20" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="E20">
         <v>0.7211</v>
@@ -842,16 +923,356 @@
       <c r="B21" t="s">
         <v>8</v>
       </c>
-      <c r="C21" t="s">
-        <v>9</v>
+      <c r="C21">
+        <v>1</v>
       </c>
       <c r="D21" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E21">
         <v>0.5838</v>
       </c>
       <c r="F21" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" t="s">
+        <v>6</v>
+      </c>
+      <c r="B22" t="s">
+        <v>9</v>
+      </c>
+      <c r="C22">
+        <v>1</v>
+      </c>
+      <c r="D22" t="s">
+        <v>40</v>
+      </c>
+      <c r="E22">
+        <v>0.6777</v>
+      </c>
+      <c r="F22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" t="s">
+        <v>6</v>
+      </c>
+      <c r="B23" t="s">
+        <v>10</v>
+      </c>
+      <c r="C23">
+        <v>1</v>
+      </c>
+      <c r="D23" t="s">
+        <v>41</v>
+      </c>
+      <c r="E23">
+        <v>0.6778999999999999</v>
+      </c>
+      <c r="F23" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" t="s">
+        <v>6</v>
+      </c>
+      <c r="B24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C24">
+        <v>1</v>
+      </c>
+      <c r="D24" t="s">
+        <v>42</v>
+      </c>
+      <c r="E24">
+        <v>0.6841</v>
+      </c>
+      <c r="F24" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
+      <c r="A25" t="s">
+        <v>6</v>
+      </c>
+      <c r="B25" t="s">
+        <v>12</v>
+      </c>
+      <c r="C25">
+        <v>1</v>
+      </c>
+      <c r="D25" t="s">
+        <v>43</v>
+      </c>
+      <c r="E25">
+        <v>0.6841</v>
+      </c>
+      <c r="F25" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
+      <c r="A26" t="s">
+        <v>6</v>
+      </c>
+      <c r="B26" t="s">
+        <v>13</v>
+      </c>
+      <c r="C26">
+        <v>1</v>
+      </c>
+      <c r="D26" t="s">
+        <v>43</v>
+      </c>
+      <c r="E26">
+        <v>0.6841</v>
+      </c>
+      <c r="F26" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
+      <c r="A27" t="s">
+        <v>6</v>
+      </c>
+      <c r="B27" t="s">
+        <v>14</v>
+      </c>
+      <c r="C27">
+        <v>1</v>
+      </c>
+      <c r="D27" t="s">
+        <v>43</v>
+      </c>
+      <c r="E27">
+        <v>0.6841</v>
+      </c>
+      <c r="F27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28" t="s">
+        <v>6</v>
+      </c>
+      <c r="B28" t="s">
+        <v>15</v>
+      </c>
+      <c r="C28">
+        <v>1</v>
+      </c>
+      <c r="D28" t="s">
+        <v>44</v>
+      </c>
+      <c r="E28">
+        <v>0.5894</v>
+      </c>
+      <c r="F28" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
+      <c r="A29" t="s">
+        <v>6</v>
+      </c>
+      <c r="B29" t="s">
+        <v>15</v>
+      </c>
+      <c r="C29">
+        <v>2</v>
+      </c>
+      <c r="D29" t="s">
+        <v>45</v>
+      </c>
+      <c r="E29">
+        <v>0.6067</v>
+      </c>
+      <c r="F29" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
+      <c r="A30" t="s">
+        <v>6</v>
+      </c>
+      <c r="B30" t="s">
+        <v>15</v>
+      </c>
+      <c r="C30">
+        <v>3</v>
+      </c>
+      <c r="D30" t="s">
+        <v>46</v>
+      </c>
+      <c r="E30">
+        <v>0.6036</v>
+      </c>
+      <c r="F30" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
+      <c r="A31" t="s">
+        <v>6</v>
+      </c>
+      <c r="B31" t="s">
+        <v>15</v>
+      </c>
+      <c r="C31">
+        <v>4</v>
+      </c>
+      <c r="D31" t="s">
+        <v>47</v>
+      </c>
+      <c r="E31">
+        <v>0.6428</v>
+      </c>
+      <c r="F31" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
+      <c r="A32" t="s">
+        <v>6</v>
+      </c>
+      <c r="B32" t="s">
+        <v>15</v>
+      </c>
+      <c r="C32">
+        <v>5</v>
+      </c>
+      <c r="D32" t="s">
+        <v>48</v>
+      </c>
+      <c r="E32">
+        <v>0.4052</v>
+      </c>
+      <c r="F32" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
+      <c r="A33" t="s">
+        <v>6</v>
+      </c>
+      <c r="B33" t="s">
+        <v>15</v>
+      </c>
+      <c r="C33">
+        <v>6</v>
+      </c>
+      <c r="D33" t="s">
+        <v>49</v>
+      </c>
+      <c r="E33">
+        <v>0.625</v>
+      </c>
+      <c r="F33" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6">
+      <c r="A34" t="s">
+        <v>6</v>
+      </c>
+      <c r="B34" t="s">
+        <v>15</v>
+      </c>
+      <c r="C34">
+        <v>7</v>
+      </c>
+      <c r="D34" t="s">
+        <v>50</v>
+      </c>
+      <c r="E34">
+        <v>0.6039</v>
+      </c>
+      <c r="F34" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6">
+      <c r="A35" t="s">
+        <v>6</v>
+      </c>
+      <c r="B35" t="s">
+        <v>16</v>
+      </c>
+      <c r="C35" t="s">
+        <v>17</v>
+      </c>
+      <c r="D35" t="s">
+        <v>51</v>
+      </c>
+      <c r="E35">
+        <v>0.6194</v>
+      </c>
+      <c r="F35" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6">
+      <c r="A36" t="s">
+        <v>6</v>
+      </c>
+      <c r="B36" t="s">
+        <v>16</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36" t="s">
+        <v>52</v>
+      </c>
+      <c r="E36">
+        <v>0.6367</v>
+      </c>
+      <c r="F36" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6">
+      <c r="A37" t="s">
+        <v>6</v>
+      </c>
+      <c r="B37" t="s">
+        <v>16</v>
+      </c>
+      <c r="C37" t="s">
+        <v>19</v>
+      </c>
+      <c r="D37" t="s">
+        <v>53</v>
+      </c>
+      <c r="E37">
+        <v>0.6216</v>
+      </c>
+      <c r="F37" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6">
+      <c r="A38" t="s">
+        <v>6</v>
+      </c>
+      <c r="B38" t="s">
+        <v>16</v>
+      </c>
+      <c r="C38" t="s">
+        <v>20</v>
+      </c>
+      <c r="D38" t="s">
+        <v>54</v>
+      </c>
+      <c r="E38">
+        <v>0.6395999999999999</v>
+      </c>
+      <c r="F38" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
UI Updates after Focus Group
</commit_message>
<xml_diff>
--- a/backend/POC/prefilter_cache.xlsx
+++ b/backend/POC/prefilter_cache.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="729" uniqueCount="201">
   <si>
     <t>process_hash</t>
   </si>
@@ -76,6 +76,15 @@
     <t>d153751413d830ba</t>
   </si>
   <si>
+    <t>c8736219f33e790f</t>
+  </si>
+  <si>
+    <t>98e721e49a3373e4</t>
+  </si>
+  <si>
+    <t>b4d05022165f08ab</t>
+  </si>
+  <si>
     <t>synthetic-compliance-rules-#1</t>
   </si>
   <si>
@@ -130,6 +139,12 @@
     <t>claude_merchant_onboarding</t>
   </si>
   <si>
+    <t>ki</t>
+  </si>
+  <si>
+    <t>ki2</t>
+  </si>
+  <si>
     <t>1</t>
   </si>
   <si>
@@ -143,6 +158,63 @@
   </si>
   <si>
     <t>5</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>24</t>
   </si>
   <si>
     <t>All payment service providers shall conduct a comprehensive identity verification of each merchant prior to granting access to payment processing services.</t>
@@ -482,6 +554,115 @@
   </si>
   <si>
     <t>21Consumer complaints must be acknowledged within two business days and resolved within 30 calendar days of receipt.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"># Datenschutz-Richtlinie_Kunstliche_Intelligenz_KI-070426-133246.pdf
+Richtlinie Künstliche Intelligenz (KI) Vorgaben und Nutzungshinweise für den Einsatz von KI / ML-Systemen mit der Beschreibung der </t>
+  </si>
+  <si>
+    <t>1    Einleitung Bei der viadee kann der Bedarf bestehen, Angebote von Künstlicher Intelligenz (KI) zu nutzen .
+Damit sind KI-Systeme im Sinne des EU Ai Acts gemeint ( ), insb. Dienste im Internet.
+Bei</t>
+  </si>
+  <si>
+    <t>1. “KI-Tools dürfen nicht allein und ohne menschliche Überprüfung, sondern ausschließlich unterstützend eingesetzt werden, wenn es um die Bewertung oder Beurteilung von Menschen geht.”</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. KI-Systeme sollen nicht mit viadee internen Informationen versorgt werden, insbesondere gilt dies für sicherheitsrelevante Informationen und für personenbezogenen Daten wenn sie im Sinne der DSGVO </t>
+  </si>
+  <si>
+    <t>3. KI-generierte Ergebnisse sollten kritisch geprüft und hinterfragt und nicht unbesehen verwendet sowie nötigenfalls gekennzeichnet werden.</t>
+  </si>
+  <si>
+    <t>4. Die viadee stellt geprüfte KI-Tools und Dienste zur Verfügung - nur diese sind zu verwenden.
+Ausnahmen zu Test- und Analysenzwecken sind nach Rücksprache mit Verantwortlichen und gegebenenfalls Bet</t>
+  </si>
+  <si>
+    <t>2    Geltungsbereich Diese Richtlinie verpflichtet alle Beschäftigten der viadee zur Einhaltung der hier festgelegten Vorgaben im Umgang mit KI- Systemen, während sie für die viadee agieren.
+Sollte im</t>
+  </si>
+  <si>
+    <t>3    Zulässigkeit des Einsatzes von KI / ML- Systemen</t>
+  </si>
+  <si>
+    <t>1. Nutzbare Software: Nur freigegebene KI-Systeme dürfen verwendet werden. Diese sind auf der Liste der explizit aufgeführt.
+Deren grundsätzliche Verwendbarkeit inklusive deren KI- Funktionen wird aus</t>
+  </si>
+  <si>
+    <t>2. Bei der Benutzung sind die dort genannten Nutzungskonzepte zu beachten.</t>
+  </si>
+  <si>
+    <t>3. Es dürfen darüber hinaus keine KI-Systeme verwendet werden, die die Eingaben von Anwender:innen, ggf.
+mitgesendete Kontextinformationen sowie die Ausgaben des KI-Systems zum Training verwenden.
+Ein</t>
+  </si>
+  <si>
+    <t>4    Verwendungseinschränkung von KI / ML- Systemen</t>
+  </si>
+  <si>
+    <t>1. Die Verwendung von a. als geheimhaltungsbedürftig eingestuften Informationen (z.B. Geschäfts- und Betriebsgeheimnisse oder sonstige Informationen, die einen besonderen wirtschaftlichen Wert für via</t>
+  </si>
+  <si>
+    <t>2. Die Nutzung eines KI-Systems zum Zweck der Erstellung von Beurteilungen der Persönlichkeit, der Arbeitsleistung, der physischen und psychischen Belastbarkeit, der kognitiven oder emotionalen Fähigk</t>
+  </si>
+  <si>
+    <t>3. Die jeweiligen KI-Tool Bedingungen sind zu beachten. Typischerweise sind diese in AGB, “Terms of Use”, “Acceptable Use” oder vergleichbaren Dokumenten zu finden.</t>
+  </si>
+  <si>
+    <t>5    Verantwortungsvoller Umgang mit KI-generierten Ergebnissen</t>
+  </si>
+  <si>
+    <t>1. Transparenz a. Wenn wir KI-Systeme betreiben, stellen wir sicher, dass sie als solche zu erkennen sind (Vgl.
+).
+b. Werden die Ergebnisse eines KI-Systems ganz oder teilweise veröffentlicht oder für</t>
+  </si>
+  <si>
+    <t>2. Da auf rein generierten Inhalten kein Urheberrecht entsteht, sind alle Inhalte manuell nachzubearbeiten, für die die viadee eine Urheberschaft anstrebt.</t>
+  </si>
+  <si>
+    <t>3. Der Dienst kann ungenaue oder falsche Informationen erstellen. Daher sind die Beschäftigten der viadee verpflichtet, die fachliche und sachliche Korrektheit der erstellten Ergebnisse durch ihr Expe</t>
+  </si>
+  <si>
+    <t>4. Ungeprüfte Arbeitsergebnisse eines KI-Tools müssen in der Kommunikation immer als solche gekennzeichnet werden.</t>
+  </si>
+  <si>
+    <t>5. Ein KI-Tool kann Ergebnisse liefern, die unter Umständen bereits urheberrechtlich geschützten Werken entsprechen. Bei Verdachtsfällen und wenn wir nicht durch den Anbieter der Software von Urheberr</t>
+  </si>
+  <si>
+    <t>6. Ein KI-Tool kann Ergebnisse liefern, die z. B. das Markenrecht, das Recht auf das eigene Bild, Verbot von Diskriminierung oder andere Gesetze zu den Ergebnistypen (Text, Bild, Audio, …) einer KI ve</t>
+  </si>
+  <si>
+    <t>6    Zum Umgang mit dieser Richtlinie Im Zweifel oder bei Unsicherheiten bei dem Einsatz eines KI-Tools oder Dienstes oder im Umgang mit den Vorgaben und Empfehlungen dieser Richtlinie sollte Rückspra</t>
+  </si>
+  <si>
+    <t>7    Aktualisierung dieser Richtlinie Die Gesetzgebung zum Thema KI hat eine hohe Dynamik und diese kann sich auf die Inhalte dieser Richtlinie auswirken. Weiterhin können z. B. neue Möglichkeiten der</t>
+  </si>
+  <si>
+    <t>1    Einleitung Bei der viadee kann der Bedarf bestehen, Angebote von Künstlicher Intelligenz (KI) zu nutzen .
+Damit sind KI-Systeme im Sinne des EU Ai Acts gemeint (hier erklärt), insb. Dienste im In</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2    Geltungsbereich Diese Richtlinie verpflichtet alle Beschäftigten der viadee zur Einhaltung der hier festgelegten Vorgaben im Umgang mit KI-Systemen, während sie für die viadee agieren.
+Sollte im </t>
+  </si>
+  <si>
+    <t>3    Zulässigkeit des Einsatzes von KI / ML-Systemen Nutzbare Software: Nur freigegebene KI-Systeme dürfen verwendet werden. Diese sind auf der Liste der KI-Anwendungen explizit aufgeführt.
+Deren grun</t>
+  </si>
+  <si>
+    <t>4    Verwendungseinschränkung von KI / ML-Systemen Die Verwendung von
+als geheimhaltungsbedürftigVerpflichtungserklärung Daten- und Geschäftsgeheimnis (Wiki-Version)eingestuften Informationen (z.B. Ge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5    Verantwortungsvoller Umgang mit KI-generierten Ergebnissen Transparenz
+Wenn wir KI-Systeme betreiben, stellen wir sicher, dass sie als solche zu erkennen sind (Vgl. EU Ai Act Artikel 50).
+Werden </t>
+  </si>
+  <si>
+    <t>6    Zum Umgang mit dieser Richtlinie Im Zweifel oder bei Unsicherheiten bei dem Einsatz eines KI-Tools oder Dienstes oder im Umgang mit den Vorgaben und Empfehlungen dieser Richtlinie sollte Rückspra</t>
+  </si>
+  <si>
+    <t>7    Aktualisierung dieser Richtlinie Die Gesetzgebung zum Thema KI hat eine hohe Dynamik und diese kann sich auf die Inhalte dieser Richtlinie auswirken. Weiterhin können z. B. neue Möglichkeiten der</t>
   </si>
 </sst>
 </file>
@@ -813,7 +994,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F174"/>
+  <dimension ref="A1:F234"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -841,13 +1022,13 @@
         <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C2">
         <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>43</v>
+        <v>67</v>
       </c>
       <c r="E2">
         <v>0.5838</v>
@@ -861,13 +1042,13 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C3">
         <v>8</v>
       </c>
       <c r="D3" t="s">
-        <v>44</v>
+        <v>68</v>
       </c>
       <c r="E3">
         <v>0.6263</v>
@@ -881,13 +1062,13 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C4">
         <v>9</v>
       </c>
       <c r="D4" t="s">
-        <v>45</v>
+        <v>69</v>
       </c>
       <c r="E4">
         <v>0.6303</v>
@@ -901,13 +1082,13 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C5">
         <v>10</v>
       </c>
       <c r="D5" t="s">
-        <v>46</v>
+        <v>70</v>
       </c>
       <c r="E5">
         <v>0.6439</v>
@@ -921,13 +1102,13 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C6">
         <v>11</v>
       </c>
       <c r="D6" t="s">
-        <v>47</v>
+        <v>71</v>
       </c>
       <c r="E6">
         <v>0.4402</v>
@@ -941,13 +1122,13 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C7">
         <v>12</v>
       </c>
       <c r="D7" t="s">
-        <v>48</v>
+        <v>72</v>
       </c>
       <c r="E7">
         <v>0.6491</v>
@@ -961,13 +1142,13 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C8">
         <v>13</v>
       </c>
       <c r="D8" t="s">
-        <v>49</v>
+        <v>73</v>
       </c>
       <c r="E8">
         <v>0.6712</v>
@@ -981,13 +1162,13 @@
         <v>6</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C9">
         <v>14</v>
       </c>
       <c r="D9" t="s">
-        <v>50</v>
+        <v>74</v>
       </c>
       <c r="E9">
         <v>0.5116000000000001</v>
@@ -1001,13 +1182,13 @@
         <v>6</v>
       </c>
       <c r="B10" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C10">
         <v>15</v>
       </c>
       <c r="D10" t="s">
-        <v>51</v>
+        <v>75</v>
       </c>
       <c r="E10">
         <v>0.5103</v>
@@ -1021,13 +1202,13 @@
         <v>6</v>
       </c>
       <c r="B11" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C11">
         <v>16</v>
       </c>
       <c r="D11" t="s">
-        <v>52</v>
+        <v>76</v>
       </c>
       <c r="E11">
         <v>0.521</v>
@@ -1041,13 +1222,13 @@
         <v>6</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C12">
         <v>17</v>
       </c>
       <c r="D12" t="s">
-        <v>53</v>
+        <v>77</v>
       </c>
       <c r="E12">
         <v>0.7005</v>
@@ -1061,13 +1242,13 @@
         <v>6</v>
       </c>
       <c r="B13" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C13">
         <v>18</v>
       </c>
       <c r="D13" t="s">
-        <v>54</v>
+        <v>78</v>
       </c>
       <c r="E13">
         <v>0.4253</v>
@@ -1081,13 +1262,13 @@
         <v>6</v>
       </c>
       <c r="B14" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C14">
         <v>19</v>
       </c>
       <c r="D14" t="s">
-        <v>55</v>
+        <v>79</v>
       </c>
       <c r="E14">
         <v>0.4379</v>
@@ -1101,13 +1282,13 @@
         <v>6</v>
       </c>
       <c r="B15" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C15">
         <v>20</v>
       </c>
       <c r="D15" t="s">
-        <v>56</v>
+        <v>80</v>
       </c>
       <c r="E15">
         <v>0.6097</v>
@@ -1121,13 +1302,13 @@
         <v>6</v>
       </c>
       <c r="B16" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C16">
         <v>21</v>
       </c>
       <c r="D16" t="s">
-        <v>57</v>
+        <v>81</v>
       </c>
       <c r="E16">
         <v>0.4384</v>
@@ -1141,13 +1322,13 @@
         <v>6</v>
       </c>
       <c r="B17" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C17">
         <v>22</v>
       </c>
       <c r="D17" t="s">
-        <v>58</v>
+        <v>82</v>
       </c>
       <c r="E17">
         <v>0.427</v>
@@ -1161,13 +1342,13 @@
         <v>6</v>
       </c>
       <c r="B18" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C18">
         <v>27</v>
       </c>
       <c r="D18" t="s">
-        <v>59</v>
+        <v>83</v>
       </c>
       <c r="E18">
         <v>0.6855</v>
@@ -1181,13 +1362,13 @@
         <v>6</v>
       </c>
       <c r="B19" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C19">
         <v>28</v>
       </c>
       <c r="D19" t="s">
-        <v>60</v>
+        <v>84</v>
       </c>
       <c r="E19">
         <v>0.5853</v>
@@ -1201,13 +1382,13 @@
         <v>6</v>
       </c>
       <c r="B20" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C20">
         <v>29</v>
       </c>
       <c r="D20" t="s">
-        <v>61</v>
+        <v>85</v>
       </c>
       <c r="E20">
         <v>0.7211</v>
@@ -1221,13 +1402,13 @@
         <v>6</v>
       </c>
       <c r="B21" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C21">
         <v>1</v>
       </c>
       <c r="D21" t="s">
-        <v>43</v>
+        <v>67</v>
       </c>
       <c r="E21">
         <v>0.5838</v>
@@ -1241,13 +1422,13 @@
         <v>6</v>
       </c>
       <c r="B22" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C22">
         <v>1</v>
       </c>
       <c r="D22" t="s">
-        <v>62</v>
+        <v>86</v>
       </c>
       <c r="E22">
         <v>0.6777</v>
@@ -1261,13 +1442,13 @@
         <v>6</v>
       </c>
       <c r="B23" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C23">
         <v>1</v>
       </c>
       <c r="D23" t="s">
-        <v>63</v>
+        <v>87</v>
       </c>
       <c r="E23">
         <v>0.6778999999999999</v>
@@ -1281,13 +1462,13 @@
         <v>6</v>
       </c>
       <c r="B24" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C24">
         <v>1</v>
       </c>
       <c r="D24" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="E24">
         <v>0.6841</v>
@@ -1301,13 +1482,13 @@
         <v>6</v>
       </c>
       <c r="B25" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C25">
         <v>1</v>
       </c>
       <c r="D25" t="s">
-        <v>65</v>
+        <v>89</v>
       </c>
       <c r="E25">
         <v>0.6841</v>
@@ -1321,13 +1502,13 @@
         <v>6</v>
       </c>
       <c r="B26" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C26">
         <v>1</v>
       </c>
       <c r="D26" t="s">
-        <v>65</v>
+        <v>89</v>
       </c>
       <c r="E26">
         <v>0.6841</v>
@@ -1341,13 +1522,13 @@
         <v>6</v>
       </c>
       <c r="B27" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C27">
         <v>1</v>
       </c>
       <c r="D27" t="s">
-        <v>65</v>
+        <v>89</v>
       </c>
       <c r="E27">
         <v>0.6841</v>
@@ -1361,13 +1542,13 @@
         <v>6</v>
       </c>
       <c r="B28" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C28">
         <v>1</v>
       </c>
       <c r="D28" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="E28">
         <v>0.5894</v>
@@ -1381,13 +1562,13 @@
         <v>6</v>
       </c>
       <c r="B29" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C29">
         <v>2</v>
       </c>
       <c r="D29" t="s">
-        <v>67</v>
+        <v>91</v>
       </c>
       <c r="E29">
         <v>0.6067</v>
@@ -1401,13 +1582,13 @@
         <v>6</v>
       </c>
       <c r="B30" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C30">
         <v>3</v>
       </c>
       <c r="D30" t="s">
-        <v>68</v>
+        <v>92</v>
       </c>
       <c r="E30">
         <v>0.6036</v>
@@ -1421,13 +1602,13 @@
         <v>6</v>
       </c>
       <c r="B31" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C31">
         <v>4</v>
       </c>
       <c r="D31" t="s">
-        <v>69</v>
+        <v>93</v>
       </c>
       <c r="E31">
         <v>0.6428</v>
@@ -1441,13 +1622,13 @@
         <v>6</v>
       </c>
       <c r="B32" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C32">
         <v>5</v>
       </c>
       <c r="D32" t="s">
-        <v>70</v>
+        <v>94</v>
       </c>
       <c r="E32">
         <v>0.4052</v>
@@ -1461,13 +1642,13 @@
         <v>6</v>
       </c>
       <c r="B33" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C33">
         <v>6</v>
       </c>
       <c r="D33" t="s">
-        <v>71</v>
+        <v>95</v>
       </c>
       <c r="E33">
         <v>0.625</v>
@@ -1481,13 +1662,13 @@
         <v>6</v>
       </c>
       <c r="B34" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C34">
         <v>7</v>
       </c>
       <c r="D34" t="s">
-        <v>72</v>
+        <v>96</v>
       </c>
       <c r="E34">
         <v>0.6039</v>
@@ -1501,13 +1682,13 @@
         <v>6</v>
       </c>
       <c r="B35" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C35">
         <v>1</v>
       </c>
       <c r="D35" t="s">
-        <v>73</v>
+        <v>97</v>
       </c>
       <c r="E35">
         <v>0.6194</v>
@@ -1521,13 +1702,13 @@
         <v>6</v>
       </c>
       <c r="B36" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C36">
         <v>2</v>
       </c>
       <c r="D36" t="s">
-        <v>74</v>
+        <v>98</v>
       </c>
       <c r="E36">
         <v>0.6367</v>
@@ -1541,13 +1722,13 @@
         <v>6</v>
       </c>
       <c r="B37" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C37">
         <v>3</v>
       </c>
       <c r="D37" t="s">
-        <v>75</v>
+        <v>99</v>
       </c>
       <c r="E37">
         <v>0.6216</v>
@@ -1561,13 +1742,13 @@
         <v>6</v>
       </c>
       <c r="B38" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C38">
         <v>4</v>
       </c>
       <c r="D38" t="s">
-        <v>76</v>
+        <v>100</v>
       </c>
       <c r="E38">
         <v>0.6395999999999999</v>
@@ -1581,13 +1762,13 @@
         <v>6</v>
       </c>
       <c r="B39" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C39">
         <v>1</v>
       </c>
       <c r="D39" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="E39">
         <v>0.6151</v>
@@ -1601,13 +1782,13 @@
         <v>6</v>
       </c>
       <c r="B40" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C40">
         <v>2</v>
       </c>
       <c r="D40" t="s">
-        <v>78</v>
+        <v>102</v>
       </c>
       <c r="E40">
         <v>0.6411</v>
@@ -1621,13 +1802,13 @@
         <v>6</v>
       </c>
       <c r="B41" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C41">
         <v>3</v>
       </c>
       <c r="D41" t="s">
-        <v>79</v>
+        <v>103</v>
       </c>
       <c r="E41">
         <v>0.4462</v>
@@ -1641,13 +1822,13 @@
         <v>6</v>
       </c>
       <c r="B42" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C42">
         <v>4</v>
       </c>
       <c r="D42" t="s">
-        <v>80</v>
+        <v>104</v>
       </c>
       <c r="E42">
         <v>0.5122</v>
@@ -1661,13 +1842,13 @@
         <v>6</v>
       </c>
       <c r="B43" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C43">
         <v>1</v>
       </c>
       <c r="D43" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="E43">
         <v>0.5894</v>
@@ -1681,13 +1862,13 @@
         <v>6</v>
       </c>
       <c r="B44" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C44">
         <v>2</v>
       </c>
       <c r="D44" t="s">
-        <v>67</v>
+        <v>91</v>
       </c>
       <c r="E44">
         <v>0.6067</v>
@@ -1701,13 +1882,13 @@
         <v>6</v>
       </c>
       <c r="B45" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C45">
         <v>3</v>
       </c>
       <c r="D45" t="s">
-        <v>68</v>
+        <v>92</v>
       </c>
       <c r="E45">
         <v>0.6036</v>
@@ -1721,13 +1902,13 @@
         <v>6</v>
       </c>
       <c r="B46" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C46">
         <v>4</v>
       </c>
       <c r="D46" t="s">
-        <v>69</v>
+        <v>93</v>
       </c>
       <c r="E46">
         <v>0.6428</v>
@@ -1741,13 +1922,13 @@
         <v>6</v>
       </c>
       <c r="B47" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C47">
         <v>5</v>
       </c>
       <c r="D47" t="s">
-        <v>70</v>
+        <v>94</v>
       </c>
       <c r="E47">
         <v>0.4052</v>
@@ -1761,13 +1942,13 @@
         <v>6</v>
       </c>
       <c r="B48" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C48">
         <v>6</v>
       </c>
       <c r="D48" t="s">
-        <v>71</v>
+        <v>95</v>
       </c>
       <c r="E48">
         <v>0.625</v>
@@ -1781,13 +1962,13 @@
         <v>6</v>
       </c>
       <c r="B49" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C49">
         <v>7</v>
       </c>
       <c r="D49" t="s">
-        <v>72</v>
+        <v>96</v>
       </c>
       <c r="E49">
         <v>0.6039</v>
@@ -1801,13 +1982,13 @@
         <v>6</v>
       </c>
       <c r="B50" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C50">
         <v>8</v>
       </c>
       <c r="D50" t="s">
-        <v>81</v>
+        <v>105</v>
       </c>
       <c r="E50">
         <v>0.4927</v>
@@ -1821,13 +2002,13 @@
         <v>7</v>
       </c>
       <c r="B51" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C51">
         <v>1</v>
       </c>
       <c r="D51" t="s">
-        <v>82</v>
+        <v>106</v>
       </c>
       <c r="E51">
         <v>0.6346000000000001</v>
@@ -1841,13 +2022,13 @@
         <v>7</v>
       </c>
       <c r="B52" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C52">
         <v>2</v>
       </c>
       <c r="D52" t="s">
-        <v>83</v>
+        <v>107</v>
       </c>
       <c r="E52">
         <v>0.3461</v>
@@ -1861,13 +2042,13 @@
         <v>7</v>
       </c>
       <c r="B53" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C53">
         <v>3</v>
       </c>
       <c r="D53" t="s">
-        <v>84</v>
+        <v>108</v>
       </c>
       <c r="E53">
         <v>0.15</v>
@@ -1881,13 +2062,13 @@
         <v>7</v>
       </c>
       <c r="B54" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C54">
         <v>4</v>
       </c>
       <c r="D54" t="s">
-        <v>85</v>
+        <v>109</v>
       </c>
       <c r="E54">
         <v>0.4212</v>
@@ -1901,13 +2082,13 @@
         <v>7</v>
       </c>
       <c r="B55" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C55">
         <v>5</v>
       </c>
       <c r="D55" t="s">
-        <v>86</v>
+        <v>110</v>
       </c>
       <c r="E55">
         <v>0.3107</v>
@@ -1921,13 +2102,13 @@
         <v>7</v>
       </c>
       <c r="B56" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C56">
         <v>6</v>
       </c>
       <c r="D56" t="s">
-        <v>87</v>
+        <v>111</v>
       </c>
       <c r="E56">
         <v>0.2965</v>
@@ -1941,13 +2122,13 @@
         <v>7</v>
       </c>
       <c r="B57" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C57">
         <v>7</v>
       </c>
       <c r="D57" t="s">
-        <v>88</v>
+        <v>112</v>
       </c>
       <c r="E57">
         <v>0.2812</v>
@@ -1961,13 +2142,13 @@
         <v>7</v>
       </c>
       <c r="B58" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C58">
         <v>8</v>
       </c>
       <c r="D58" t="s">
-        <v>89</v>
+        <v>113</v>
       </c>
       <c r="E58">
         <v>0.2349</v>
@@ -1981,13 +2162,13 @@
         <v>7</v>
       </c>
       <c r="B59" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C59">
         <v>9</v>
       </c>
       <c r="D59" t="s">
-        <v>90</v>
+        <v>114</v>
       </c>
       <c r="E59">
         <v>0.6031</v>
@@ -2001,13 +2182,13 @@
         <v>7</v>
       </c>
       <c r="B60" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C60">
         <v>10</v>
       </c>
       <c r="D60" t="s">
-        <v>91</v>
+        <v>115</v>
       </c>
       <c r="E60">
         <v>0.4668</v>
@@ -2021,13 +2202,13 @@
         <v>8</v>
       </c>
       <c r="B61" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C61">
         <v>1</v>
       </c>
       <c r="D61" t="s">
-        <v>92</v>
+        <v>116</v>
       </c>
       <c r="E61">
         <v>0.4043</v>
@@ -2041,13 +2222,13 @@
         <v>8</v>
       </c>
       <c r="B62" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C62">
         <v>2</v>
       </c>
       <c r="D62" t="s">
-        <v>93</v>
+        <v>117</v>
       </c>
       <c r="E62">
         <v>0.496</v>
@@ -2061,13 +2242,13 @@
         <v>8</v>
       </c>
       <c r="B63" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C63">
         <v>3</v>
       </c>
       <c r="D63" t="s">
-        <v>94</v>
+        <v>118</v>
       </c>
       <c r="E63">
         <v>0.4781</v>
@@ -2081,13 +2262,13 @@
         <v>8</v>
       </c>
       <c r="B64" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C64">
         <v>4</v>
       </c>
       <c r="D64" t="s">
-        <v>95</v>
+        <v>119</v>
       </c>
       <c r="E64">
         <v>0.5125</v>
@@ -2101,13 +2282,13 @@
         <v>8</v>
       </c>
       <c r="B65" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C65">
         <v>5</v>
       </c>
       <c r="D65" t="s">
-        <v>96</v>
+        <v>120</v>
       </c>
       <c r="E65">
         <v>0.3548</v>
@@ -2121,13 +2302,13 @@
         <v>8</v>
       </c>
       <c r="B66" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C66">
         <v>6</v>
       </c>
       <c r="D66" t="s">
-        <v>97</v>
+        <v>121</v>
       </c>
       <c r="E66">
         <v>0.2212</v>
@@ -2141,13 +2322,13 @@
         <v>8</v>
       </c>
       <c r="B67" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C67">
         <v>7</v>
       </c>
       <c r="D67" t="s">
-        <v>98</v>
+        <v>122</v>
       </c>
       <c r="E67">
         <v>0.3205</v>
@@ -2161,13 +2342,13 @@
         <v>8</v>
       </c>
       <c r="B68" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C68">
         <v>8</v>
       </c>
       <c r="D68" t="s">
-        <v>99</v>
+        <v>123</v>
       </c>
       <c r="E68">
         <v>0.2504</v>
@@ -2181,13 +2362,13 @@
         <v>8</v>
       </c>
       <c r="B69" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C69">
         <v>9</v>
       </c>
       <c r="D69" t="s">
-        <v>100</v>
+        <v>124</v>
       </c>
       <c r="E69">
         <v>0.51</v>
@@ -2201,13 +2382,13 @@
         <v>8</v>
       </c>
       <c r="B70" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C70">
         <v>10</v>
       </c>
       <c r="D70" t="s">
-        <v>101</v>
+        <v>125</v>
       </c>
       <c r="E70">
         <v>0.4057</v>
@@ -2221,13 +2402,13 @@
         <v>9</v>
       </c>
       <c r="B71" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C71">
         <v>1</v>
       </c>
       <c r="D71" t="s">
-        <v>92</v>
+        <v>116</v>
       </c>
       <c r="E71">
         <v>0.6163999999999999</v>
@@ -2241,13 +2422,13 @@
         <v>9</v>
       </c>
       <c r="B72" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C72">
         <v>2</v>
       </c>
       <c r="D72" t="s">
-        <v>93</v>
+        <v>117</v>
       </c>
       <c r="E72">
         <v>0.5685</v>
@@ -2261,13 +2442,13 @@
         <v>9</v>
       </c>
       <c r="B73" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C73">
         <v>3</v>
       </c>
       <c r="D73" t="s">
-        <v>94</v>
+        <v>118</v>
       </c>
       <c r="E73">
         <v>0.6151</v>
@@ -2281,13 +2462,13 @@
         <v>9</v>
       </c>
       <c r="B74" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C74">
         <v>4</v>
       </c>
       <c r="D74" t="s">
-        <v>95</v>
+        <v>119</v>
       </c>
       <c r="E74">
         <v>0.6232</v>
@@ -2301,13 +2482,13 @@
         <v>9</v>
       </c>
       <c r="B75" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C75">
         <v>5</v>
       </c>
       <c r="D75" t="s">
-        <v>96</v>
+        <v>120</v>
       </c>
       <c r="E75">
         <v>0.5322</v>
@@ -2321,13 +2502,13 @@
         <v>9</v>
       </c>
       <c r="B76" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C76">
         <v>6</v>
       </c>
       <c r="D76" t="s">
-        <v>97</v>
+        <v>121</v>
       </c>
       <c r="E76">
         <v>0.3512</v>
@@ -2341,13 +2522,13 @@
         <v>9</v>
       </c>
       <c r="B77" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C77">
         <v>7</v>
       </c>
       <c r="D77" t="s">
-        <v>98</v>
+        <v>122</v>
       </c>
       <c r="E77">
         <v>0.4761</v>
@@ -2361,13 +2542,13 @@
         <v>9</v>
       </c>
       <c r="B78" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C78">
         <v>8</v>
       </c>
       <c r="D78" t="s">
-        <v>99</v>
+        <v>123</v>
       </c>
       <c r="E78">
         <v>0.481</v>
@@ -2381,13 +2562,13 @@
         <v>9</v>
       </c>
       <c r="B79" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C79">
         <v>9</v>
       </c>
       <c r="D79" t="s">
-        <v>100</v>
+        <v>124</v>
       </c>
       <c r="E79">
         <v>0.5723</v>
@@ -2401,13 +2582,13 @@
         <v>9</v>
       </c>
       <c r="B80" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C80">
         <v>10</v>
       </c>
       <c r="D80" t="s">
-        <v>101</v>
+        <v>125</v>
       </c>
       <c r="E80">
         <v>0.6477000000000001</v>
@@ -2421,13 +2602,13 @@
         <v>10</v>
       </c>
       <c r="B81" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C81">
         <v>1</v>
       </c>
       <c r="D81" t="s">
-        <v>102</v>
+        <v>126</v>
       </c>
       <c r="E81">
         <v>0.4285</v>
@@ -2441,13 +2622,13 @@
         <v>10</v>
       </c>
       <c r="B82" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C82">
         <v>2</v>
       </c>
       <c r="D82" t="s">
-        <v>103</v>
+        <v>127</v>
       </c>
       <c r="E82">
         <v>0.5831</v>
@@ -2461,13 +2642,13 @@
         <v>10</v>
       </c>
       <c r="B83" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C83">
         <v>3</v>
       </c>
       <c r="D83" t="s">
-        <v>104</v>
+        <v>128</v>
       </c>
       <c r="E83">
         <v>0.3756</v>
@@ -2481,13 +2662,13 @@
         <v>10</v>
       </c>
       <c r="B84" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C84">
         <v>4</v>
       </c>
       <c r="D84" t="s">
-        <v>105</v>
+        <v>129</v>
       </c>
       <c r="E84">
         <v>0.4707</v>
@@ -2501,13 +2682,13 @@
         <v>10</v>
       </c>
       <c r="B85" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C85">
         <v>5</v>
       </c>
       <c r="D85" t="s">
-        <v>106</v>
+        <v>130</v>
       </c>
       <c r="E85">
         <v>0.4945</v>
@@ -2521,13 +2702,13 @@
         <v>10</v>
       </c>
       <c r="B86" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C86">
         <v>6</v>
       </c>
       <c r="D86" t="s">
-        <v>107</v>
+        <v>131</v>
       </c>
       <c r="E86">
         <v>0.3551</v>
@@ -2541,13 +2722,13 @@
         <v>10</v>
       </c>
       <c r="B87" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C87">
         <v>7</v>
       </c>
       <c r="D87" t="s">
-        <v>108</v>
+        <v>132</v>
       </c>
       <c r="E87">
         <v>0.5426</v>
@@ -2561,13 +2742,13 @@
         <v>10</v>
       </c>
       <c r="B88" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C88">
         <v>8</v>
       </c>
       <c r="D88" t="s">
-        <v>109</v>
+        <v>133</v>
       </c>
       <c r="E88">
         <v>0.5185999999999999</v>
@@ -2581,13 +2762,13 @@
         <v>10</v>
       </c>
       <c r="B89" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C89">
         <v>9</v>
       </c>
       <c r="D89" t="s">
-        <v>110</v>
+        <v>134</v>
       </c>
       <c r="E89">
         <v>0.3634</v>
@@ -2601,13 +2782,13 @@
         <v>10</v>
       </c>
       <c r="B90" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C90">
         <v>10</v>
       </c>
       <c r="D90" t="s">
-        <v>111</v>
+        <v>135</v>
       </c>
       <c r="E90">
         <v>0.4161</v>
@@ -2621,13 +2802,13 @@
         <v>10</v>
       </c>
       <c r="B91" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C91">
         <v>11</v>
       </c>
       <c r="D91" t="s">
-        <v>112</v>
+        <v>136</v>
       </c>
       <c r="E91">
         <v>0.2871</v>
@@ -2641,13 +2822,13 @@
         <v>10</v>
       </c>
       <c r="B92" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C92">
         <v>12</v>
       </c>
       <c r="D92" t="s">
-        <v>113</v>
+        <v>137</v>
       </c>
       <c r="E92">
         <v>0.506</v>
@@ -2661,13 +2842,13 @@
         <v>10</v>
       </c>
       <c r="B93" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C93">
         <v>13</v>
       </c>
       <c r="D93" t="s">
-        <v>114</v>
+        <v>138</v>
       </c>
       <c r="E93">
         <v>0.4668</v>
@@ -2681,13 +2862,13 @@
         <v>10</v>
       </c>
       <c r="B94" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C94">
         <v>14</v>
       </c>
       <c r="D94" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="E94">
         <v>0.3633</v>
@@ -2701,13 +2882,13 @@
         <v>10</v>
       </c>
       <c r="B95" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C95">
         <v>15</v>
       </c>
       <c r="D95" t="s">
-        <v>116</v>
+        <v>140</v>
       </c>
       <c r="E95">
         <v>0.3922</v>
@@ -2721,13 +2902,13 @@
         <v>10</v>
       </c>
       <c r="B96" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C96">
         <v>16</v>
       </c>
       <c r="D96" t="s">
-        <v>117</v>
+        <v>141</v>
       </c>
       <c r="E96">
         <v>0.4302</v>
@@ -2741,13 +2922,13 @@
         <v>10</v>
       </c>
       <c r="B97" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C97">
         <v>17</v>
       </c>
       <c r="D97" t="s">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="E97">
         <v>0.4779</v>
@@ -2761,13 +2942,13 @@
         <v>10</v>
       </c>
       <c r="B98" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C98">
         <v>18</v>
       </c>
       <c r="D98" t="s">
-        <v>119</v>
+        <v>143</v>
       </c>
       <c r="E98">
         <v>0.4652</v>
@@ -2781,13 +2962,13 @@
         <v>10</v>
       </c>
       <c r="B99" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C99">
         <v>19</v>
       </c>
       <c r="D99" t="s">
-        <v>120</v>
+        <v>144</v>
       </c>
       <c r="E99">
         <v>0.4672</v>
@@ -2801,13 +2982,13 @@
         <v>10</v>
       </c>
       <c r="B100" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C100">
         <v>20</v>
       </c>
       <c r="D100" t="s">
-        <v>121</v>
+        <v>145</v>
       </c>
       <c r="E100">
         <v>0.4137</v>
@@ -2821,13 +3002,13 @@
         <v>10</v>
       </c>
       <c r="B101" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C101">
         <v>21</v>
       </c>
       <c r="D101" t="s">
-        <v>122</v>
+        <v>146</v>
       </c>
       <c r="E101">
         <v>0.3759</v>
@@ -2841,13 +3022,13 @@
         <v>10</v>
       </c>
       <c r="B102" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C102">
         <v>22</v>
       </c>
       <c r="D102" t="s">
-        <v>123</v>
+        <v>147</v>
       </c>
       <c r="E102">
         <v>0.3841</v>
@@ -2861,13 +3042,13 @@
         <v>10</v>
       </c>
       <c r="B103" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C103">
         <v>23</v>
       </c>
       <c r="D103" t="s">
-        <v>124</v>
+        <v>148</v>
       </c>
       <c r="E103">
         <v>0.377</v>
@@ -2881,13 +3062,13 @@
         <v>11</v>
       </c>
       <c r="B104" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C104">
         <v>1</v>
       </c>
       <c r="D104" t="s">
-        <v>125</v>
+        <v>149</v>
       </c>
       <c r="E104">
         <v>0.589</v>
@@ -2901,13 +3082,13 @@
         <v>11</v>
       </c>
       <c r="B105" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C105">
         <v>2</v>
       </c>
       <c r="D105" t="s">
-        <v>126</v>
+        <v>150</v>
       </c>
       <c r="E105">
         <v>0.5769</v>
@@ -2921,13 +3102,13 @@
         <v>11</v>
       </c>
       <c r="B106" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C106">
         <v>3</v>
       </c>
       <c r="D106" t="s">
-        <v>127</v>
+        <v>151</v>
       </c>
       <c r="E106">
         <v>0.8023</v>
@@ -2941,13 +3122,13 @@
         <v>11</v>
       </c>
       <c r="B107" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C107">
         <v>4</v>
       </c>
       <c r="D107" t="s">
-        <v>128</v>
+        <v>152</v>
       </c>
       <c r="E107">
         <v>0.6107</v>
@@ -2961,13 +3142,13 @@
         <v>11</v>
       </c>
       <c r="B108" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C108">
         <v>5</v>
       </c>
       <c r="D108" t="s">
-        <v>129</v>
+        <v>153</v>
       </c>
       <c r="E108">
         <v>0.5578</v>
@@ -2981,13 +3162,13 @@
         <v>12</v>
       </c>
       <c r="B109" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C109">
         <v>1</v>
       </c>
       <c r="D109" t="s">
-        <v>130</v>
+        <v>154</v>
       </c>
       <c r="E109">
         <v>0.525</v>
@@ -3001,13 +3182,13 @@
         <v>12</v>
       </c>
       <c r="B110" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C110">
         <v>2</v>
       </c>
       <c r="D110" t="s">
-        <v>131</v>
+        <v>155</v>
       </c>
       <c r="E110">
         <v>0.6331</v>
@@ -3021,13 +3202,13 @@
         <v>12</v>
       </c>
       <c r="B111" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C111">
         <v>3</v>
       </c>
       <c r="D111" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="E111">
         <v>0.6157</v>
@@ -3041,13 +3222,13 @@
         <v>12</v>
       </c>
       <c r="B112" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C112">
         <v>4</v>
       </c>
       <c r="D112" t="s">
-        <v>133</v>
+        <v>157</v>
       </c>
       <c r="E112">
         <v>0.5907</v>
@@ -3061,13 +3242,13 @@
         <v>12</v>
       </c>
       <c r="B113" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C113">
         <v>5</v>
       </c>
       <c r="D113" t="s">
-        <v>134</v>
+        <v>158</v>
       </c>
       <c r="E113">
         <v>0.5887</v>
@@ -3081,13 +3262,13 @@
         <v>13</v>
       </c>
       <c r="B114" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C114">
         <v>1</v>
       </c>
       <c r="D114" t="s">
-        <v>92</v>
+        <v>116</v>
       </c>
       <c r="E114">
         <v>0.4681</v>
@@ -3101,13 +3282,13 @@
         <v>13</v>
       </c>
       <c r="B115" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C115">
         <v>2</v>
       </c>
       <c r="D115" t="s">
-        <v>93</v>
+        <v>117</v>
       </c>
       <c r="E115">
         <v>0.5196</v>
@@ -3121,13 +3302,13 @@
         <v>13</v>
       </c>
       <c r="B116" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C116">
         <v>3</v>
       </c>
       <c r="D116" t="s">
-        <v>94</v>
+        <v>118</v>
       </c>
       <c r="E116">
         <v>0.4807</v>
@@ -3141,13 +3322,13 @@
         <v>13</v>
       </c>
       <c r="B117" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C117">
         <v>4</v>
       </c>
       <c r="D117" t="s">
-        <v>95</v>
+        <v>119</v>
       </c>
       <c r="E117">
         <v>0.5272</v>
@@ -3161,13 +3342,13 @@
         <v>13</v>
       </c>
       <c r="B118" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C118">
         <v>5</v>
       </c>
       <c r="D118" t="s">
-        <v>96</v>
+        <v>120</v>
       </c>
       <c r="E118">
         <v>0.4035</v>
@@ -3181,13 +3362,13 @@
         <v>13</v>
       </c>
       <c r="B119" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C119">
         <v>6</v>
       </c>
       <c r="D119" t="s">
-        <v>97</v>
+        <v>121</v>
       </c>
       <c r="E119">
         <v>0.2197</v>
@@ -3201,13 +3382,13 @@
         <v>13</v>
       </c>
       <c r="B120" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C120">
         <v>7</v>
       </c>
       <c r="D120" t="s">
-        <v>98</v>
+        <v>122</v>
       </c>
       <c r="E120">
         <v>0.3409</v>
@@ -3221,13 +3402,13 @@
         <v>13</v>
       </c>
       <c r="B121" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C121">
         <v>8</v>
       </c>
       <c r="D121" t="s">
-        <v>99</v>
+        <v>123</v>
       </c>
       <c r="E121">
         <v>0.306</v>
@@ -3241,13 +3422,13 @@
         <v>13</v>
       </c>
       <c r="B122" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C122">
         <v>9</v>
       </c>
       <c r="D122" t="s">
-        <v>100</v>
+        <v>124</v>
       </c>
       <c r="E122">
         <v>0.5057</v>
@@ -3261,13 +3442,13 @@
         <v>13</v>
       </c>
       <c r="B123" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C123">
         <v>10</v>
       </c>
       <c r="D123" t="s">
-        <v>101</v>
+        <v>125</v>
       </c>
       <c r="E123">
         <v>0.391</v>
@@ -3281,13 +3462,13 @@
         <v>14</v>
       </c>
       <c r="B124" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C124">
         <v>1</v>
       </c>
       <c r="D124" t="s">
-        <v>92</v>
+        <v>116</v>
       </c>
       <c r="E124">
         <v>0.4744</v>
@@ -3301,13 +3482,13 @@
         <v>14</v>
       </c>
       <c r="B125" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C125">
         <v>2</v>
       </c>
       <c r="D125" t="s">
-        <v>93</v>
+        <v>117</v>
       </c>
       <c r="E125">
         <v>0.5164</v>
@@ -3321,13 +3502,13 @@
         <v>14</v>
       </c>
       <c r="B126" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C126">
         <v>3</v>
       </c>
       <c r="D126" t="s">
-        <v>94</v>
+        <v>118</v>
       </c>
       <c r="E126">
         <v>0.4936</v>
@@ -3341,13 +3522,13 @@
         <v>14</v>
       </c>
       <c r="B127" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C127">
         <v>4</v>
       </c>
       <c r="D127" t="s">
-        <v>95</v>
+        <v>119</v>
       </c>
       <c r="E127">
         <v>0.5272</v>
@@ -3361,13 +3542,13 @@
         <v>14</v>
       </c>
       <c r="B128" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C128">
         <v>5</v>
       </c>
       <c r="D128" t="s">
-        <v>96</v>
+        <v>120</v>
       </c>
       <c r="E128">
         <v>0.3482</v>
@@ -3381,13 +3562,13 @@
         <v>14</v>
       </c>
       <c r="B129" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C129">
         <v>6</v>
       </c>
       <c r="D129" t="s">
-        <v>97</v>
+        <v>121</v>
       </c>
       <c r="E129">
         <v>0.2297</v>
@@ -3401,13 +3582,13 @@
         <v>14</v>
       </c>
       <c r="B130" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C130">
         <v>7</v>
       </c>
       <c r="D130" t="s">
-        <v>98</v>
+        <v>122</v>
       </c>
       <c r="E130">
         <v>0.3378</v>
@@ -3421,13 +3602,13 @@
         <v>14</v>
       </c>
       <c r="B131" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C131">
         <v>8</v>
       </c>
       <c r="D131" t="s">
-        <v>99</v>
+        <v>123</v>
       </c>
       <c r="E131">
         <v>0.3239</v>
@@ -3441,13 +3622,13 @@
         <v>14</v>
       </c>
       <c r="B132" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C132">
         <v>9</v>
       </c>
       <c r="D132" t="s">
-        <v>100</v>
+        <v>124</v>
       </c>
       <c r="E132">
         <v>0.5134</v>
@@ -3461,13 +3642,13 @@
         <v>14</v>
       </c>
       <c r="B133" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C133">
         <v>10</v>
       </c>
       <c r="D133" t="s">
-        <v>101</v>
+        <v>125</v>
       </c>
       <c r="E133">
         <v>0.4012</v>
@@ -3481,13 +3662,13 @@
         <v>15</v>
       </c>
       <c r="B134" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C134">
         <v>1</v>
       </c>
       <c r="D134" t="s">
-        <v>92</v>
+        <v>116</v>
       </c>
       <c r="E134">
         <v>0.4637</v>
@@ -3501,13 +3682,13 @@
         <v>15</v>
       </c>
       <c r="B135" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C135">
         <v>2</v>
       </c>
       <c r="D135" t="s">
-        <v>93</v>
+        <v>117</v>
       </c>
       <c r="E135">
         <v>0.5274</v>
@@ -3521,13 +3702,13 @@
         <v>15</v>
       </c>
       <c r="B136" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C136">
         <v>3</v>
       </c>
       <c r="D136" t="s">
-        <v>94</v>
+        <v>118</v>
       </c>
       <c r="E136">
         <v>0.466</v>
@@ -3541,13 +3722,13 @@
         <v>15</v>
       </c>
       <c r="B137" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C137">
         <v>4</v>
       </c>
       <c r="D137" t="s">
-        <v>95</v>
+        <v>119</v>
       </c>
       <c r="E137">
         <v>0.4992</v>
@@ -3561,13 +3742,13 @@
         <v>15</v>
       </c>
       <c r="B138" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C138">
         <v>5</v>
       </c>
       <c r="D138" t="s">
-        <v>96</v>
+        <v>120</v>
       </c>
       <c r="E138">
         <v>0.3147</v>
@@ -3581,13 +3762,13 @@
         <v>15</v>
       </c>
       <c r="B139" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C139">
         <v>6</v>
       </c>
       <c r="D139" t="s">
-        <v>97</v>
+        <v>121</v>
       </c>
       <c r="E139">
         <v>0.2325</v>
@@ -3601,13 +3782,13 @@
         <v>15</v>
       </c>
       <c r="B140" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C140">
         <v>7</v>
       </c>
       <c r="D140" t="s">
-        <v>98</v>
+        <v>122</v>
       </c>
       <c r="E140">
         <v>0.3077</v>
@@ -3621,13 +3802,13 @@
         <v>15</v>
       </c>
       <c r="B141" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C141">
         <v>8</v>
       </c>
       <c r="D141" t="s">
-        <v>99</v>
+        <v>123</v>
       </c>
       <c r="E141">
         <v>0.3327</v>
@@ -3641,13 +3822,13 @@
         <v>15</v>
       </c>
       <c r="B142" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C142">
         <v>9</v>
       </c>
       <c r="D142" t="s">
-        <v>100</v>
+        <v>124</v>
       </c>
       <c r="E142">
         <v>0.5164</v>
@@ -3661,13 +3842,13 @@
         <v>15</v>
       </c>
       <c r="B143" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C143">
         <v>10</v>
       </c>
       <c r="D143" t="s">
-        <v>101</v>
+        <v>125</v>
       </c>
       <c r="E143">
         <v>0.4241</v>
@@ -3681,13 +3862,13 @@
         <v>6</v>
       </c>
       <c r="B144" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C144">
         <v>1</v>
       </c>
       <c r="D144" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="E144">
         <v>0.5915</v>
@@ -3701,13 +3882,13 @@
         <v>6</v>
       </c>
       <c r="B145" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C145">
         <v>2</v>
       </c>
       <c r="D145" t="s">
-        <v>136</v>
+        <v>160</v>
       </c>
       <c r="E145">
         <v>0.594</v>
@@ -3721,13 +3902,13 @@
         <v>6</v>
       </c>
       <c r="B146" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C146">
         <v>3</v>
       </c>
       <c r="D146" t="s">
-        <v>137</v>
+        <v>161</v>
       </c>
       <c r="E146">
         <v>0.6373</v>
@@ -3741,13 +3922,13 @@
         <v>6</v>
       </c>
       <c r="B147" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C147">
         <v>4</v>
       </c>
       <c r="D147" t="s">
-        <v>138</v>
+        <v>162</v>
       </c>
       <c r="E147">
         <v>0.7056</v>
@@ -3761,13 +3942,13 @@
         <v>6</v>
       </c>
       <c r="B148" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C148">
         <v>5</v>
       </c>
       <c r="D148" t="s">
-        <v>139</v>
+        <v>163</v>
       </c>
       <c r="E148">
         <v>0.6233</v>
@@ -3781,13 +3962,13 @@
         <v>6</v>
       </c>
       <c r="B149" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C149">
         <v>6</v>
       </c>
       <c r="D149" t="s">
-        <v>140</v>
+        <v>164</v>
       </c>
       <c r="E149">
         <v>0.5113</v>
@@ -3801,13 +3982,13 @@
         <v>6</v>
       </c>
       <c r="B150" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C150">
         <v>7</v>
       </c>
       <c r="D150" t="s">
-        <v>141</v>
+        <v>165</v>
       </c>
       <c r="E150">
         <v>0.3871</v>
@@ -3821,13 +4002,13 @@
         <v>6</v>
       </c>
       <c r="B151" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C151">
         <v>8</v>
       </c>
       <c r="D151" t="s">
-        <v>142</v>
+        <v>166</v>
       </c>
       <c r="E151">
         <v>0.375</v>
@@ -3841,13 +4022,13 @@
         <v>6</v>
       </c>
       <c r="B152" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C152">
         <v>9</v>
       </c>
       <c r="D152" t="s">
-        <v>143</v>
+        <v>167</v>
       </c>
       <c r="E152">
         <v>0.4379</v>
@@ -3861,13 +4042,13 @@
         <v>6</v>
       </c>
       <c r="B153" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C153">
         <v>10</v>
       </c>
       <c r="D153" t="s">
-        <v>144</v>
+        <v>168</v>
       </c>
       <c r="E153">
         <v>0.5532</v>
@@ -3881,13 +4062,13 @@
         <v>6</v>
       </c>
       <c r="B154" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C154">
         <v>11</v>
       </c>
       <c r="D154" t="s">
-        <v>145</v>
+        <v>169</v>
       </c>
       <c r="E154">
         <v>0.3674</v>
@@ -3901,13 +4082,13 @@
         <v>16</v>
       </c>
       <c r="B155" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C155">
         <v>1</v>
       </c>
       <c r="D155" t="s">
-        <v>125</v>
+        <v>149</v>
       </c>
       <c r="E155">
         <v>0.5351</v>
@@ -3921,13 +4102,13 @@
         <v>16</v>
       </c>
       <c r="B156" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C156">
         <v>2</v>
       </c>
       <c r="D156" t="s">
-        <v>126</v>
+        <v>150</v>
       </c>
       <c r="E156">
         <v>0.5658</v>
@@ -3941,13 +4122,13 @@
         <v>16</v>
       </c>
       <c r="B157" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C157">
         <v>3</v>
       </c>
       <c r="D157" t="s">
-        <v>127</v>
+        <v>151</v>
       </c>
       <c r="E157">
         <v>0.8372000000000001</v>
@@ -3961,13 +4142,13 @@
         <v>16</v>
       </c>
       <c r="B158" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C158">
         <v>4</v>
       </c>
       <c r="D158" t="s">
-        <v>128</v>
+        <v>152</v>
       </c>
       <c r="E158">
         <v>0.6856</v>
@@ -3981,13 +4162,13 @@
         <v>16</v>
       </c>
       <c r="B159" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C159">
         <v>5</v>
       </c>
       <c r="D159" t="s">
-        <v>129</v>
+        <v>153</v>
       </c>
       <c r="E159">
         <v>0.4722</v>
@@ -4001,13 +4182,13 @@
         <v>17</v>
       </c>
       <c r="B160" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C160">
         <v>1</v>
       </c>
       <c r="D160" t="s">
-        <v>125</v>
+        <v>149</v>
       </c>
       <c r="E160">
         <v>0.5958</v>
@@ -4021,13 +4202,13 @@
         <v>17</v>
       </c>
       <c r="B161" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C161">
         <v>2</v>
       </c>
       <c r="D161" t="s">
-        <v>126</v>
+        <v>150</v>
       </c>
       <c r="E161">
         <v>0.5648</v>
@@ -4041,13 +4222,13 @@
         <v>17</v>
       </c>
       <c r="B162" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C162">
         <v>3</v>
       </c>
       <c r="D162" t="s">
-        <v>127</v>
+        <v>151</v>
       </c>
       <c r="E162">
         <v>0.8122</v>
@@ -4061,13 +4242,13 @@
         <v>17</v>
       </c>
       <c r="B163" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C163">
         <v>4</v>
       </c>
       <c r="D163" t="s">
-        <v>128</v>
+        <v>152</v>
       </c>
       <c r="E163">
         <v>0.5341</v>
@@ -4081,13 +4262,13 @@
         <v>17</v>
       </c>
       <c r="B164" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C164">
         <v>5</v>
       </c>
       <c r="D164" t="s">
-        <v>129</v>
+        <v>153</v>
       </c>
       <c r="E164">
         <v>0.4946</v>
@@ -4101,13 +4282,13 @@
         <v>18</v>
       </c>
       <c r="B165" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C165">
         <v>1</v>
       </c>
       <c r="D165" t="s">
-        <v>125</v>
+        <v>149</v>
       </c>
       <c r="E165">
         <v>0.45</v>
@@ -4121,13 +4302,13 @@
         <v>18</v>
       </c>
       <c r="B166" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C166">
         <v>2</v>
       </c>
       <c r="D166" t="s">
-        <v>126</v>
+        <v>150</v>
       </c>
       <c r="E166">
         <v>0.4242</v>
@@ -4141,13 +4322,13 @@
         <v>18</v>
       </c>
       <c r="B167" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C167">
         <v>3</v>
       </c>
       <c r="D167" t="s">
-        <v>127</v>
+        <v>151</v>
       </c>
       <c r="E167">
         <v>0.6752</v>
@@ -4161,13 +4342,13 @@
         <v>18</v>
       </c>
       <c r="B168" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C168">
         <v>4</v>
       </c>
       <c r="D168" t="s">
-        <v>128</v>
+        <v>152</v>
       </c>
       <c r="E168">
         <v>0.4821</v>
@@ -4181,13 +4362,13 @@
         <v>18</v>
       </c>
       <c r="B169" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C169">
         <v>5</v>
       </c>
       <c r="D169" t="s">
-        <v>129</v>
+        <v>153</v>
       </c>
       <c r="E169">
         <v>0.4399</v>
@@ -4201,13 +4382,13 @@
         <v>19</v>
       </c>
       <c r="B170" t="s">
-        <v>35</v>
-      </c>
-      <c r="C170" t="s">
         <v>38</v>
       </c>
+      <c r="C170">
+        <v>1</v>
+      </c>
       <c r="D170" t="s">
-        <v>125</v>
+        <v>149</v>
       </c>
       <c r="E170">
         <v>0.5006</v>
@@ -4221,13 +4402,13 @@
         <v>19</v>
       </c>
       <c r="B171" t="s">
-        <v>35</v>
-      </c>
-      <c r="C171" t="s">
-        <v>39</v>
+        <v>38</v>
+      </c>
+      <c r="C171">
+        <v>2</v>
       </c>
       <c r="D171" t="s">
-        <v>126</v>
+        <v>150</v>
       </c>
       <c r="E171">
         <v>0.5268</v>
@@ -4241,13 +4422,13 @@
         <v>19</v>
       </c>
       <c r="B172" t="s">
-        <v>35</v>
-      </c>
-      <c r="C172" t="s">
-        <v>40</v>
+        <v>38</v>
+      </c>
+      <c r="C172">
+        <v>3</v>
       </c>
       <c r="D172" t="s">
-        <v>127</v>
+        <v>151</v>
       </c>
       <c r="E172">
         <v>0.8122</v>
@@ -4261,13 +4442,13 @@
         <v>19</v>
       </c>
       <c r="B173" t="s">
-        <v>35</v>
-      </c>
-      <c r="C173" t="s">
-        <v>41</v>
+        <v>38</v>
+      </c>
+      <c r="C173">
+        <v>4</v>
       </c>
       <c r="D173" t="s">
-        <v>128</v>
+        <v>152</v>
       </c>
       <c r="E173">
         <v>0.5647</v>
@@ -4281,19 +4462,1219 @@
         <v>19</v>
       </c>
       <c r="B174" t="s">
-        <v>35</v>
-      </c>
-      <c r="C174" t="s">
-        <v>42</v>
+        <v>38</v>
+      </c>
+      <c r="C174">
+        <v>5</v>
       </c>
       <c r="D174" t="s">
-        <v>129</v>
+        <v>153</v>
       </c>
       <c r="E174">
         <v>0.4946</v>
       </c>
       <c r="F174" t="b">
         <v>1</v>
+      </c>
+    </row>
+    <row r="175" spans="1:6">
+      <c r="A175" t="s">
+        <v>20</v>
+      </c>
+      <c r="B175" t="s">
+        <v>38</v>
+      </c>
+      <c r="C175">
+        <v>1</v>
+      </c>
+      <c r="D175" t="s">
+        <v>149</v>
+      </c>
+      <c r="E175">
+        <v>0.4608</v>
+      </c>
+      <c r="F175" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="176" spans="1:6">
+      <c r="A176" t="s">
+        <v>20</v>
+      </c>
+      <c r="B176" t="s">
+        <v>38</v>
+      </c>
+      <c r="C176">
+        <v>2</v>
+      </c>
+      <c r="D176" t="s">
+        <v>150</v>
+      </c>
+      <c r="E176">
+        <v>0.6103</v>
+      </c>
+      <c r="F176" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="177" spans="1:6">
+      <c r="A177" t="s">
+        <v>20</v>
+      </c>
+      <c r="B177" t="s">
+        <v>38</v>
+      </c>
+      <c r="C177">
+        <v>3</v>
+      </c>
+      <c r="D177" t="s">
+        <v>151</v>
+      </c>
+      <c r="E177">
+        <v>0.6756</v>
+      </c>
+      <c r="F177" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="178" spans="1:6">
+      <c r="A178" t="s">
+        <v>20</v>
+      </c>
+      <c r="B178" t="s">
+        <v>38</v>
+      </c>
+      <c r="C178">
+        <v>4</v>
+      </c>
+      <c r="D178" t="s">
+        <v>152</v>
+      </c>
+      <c r="E178">
+        <v>0.5163</v>
+      </c>
+      <c r="F178" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="179" spans="1:6">
+      <c r="A179" t="s">
+        <v>20</v>
+      </c>
+      <c r="B179" t="s">
+        <v>38</v>
+      </c>
+      <c r="C179">
+        <v>5</v>
+      </c>
+      <c r="D179" t="s">
+        <v>153</v>
+      </c>
+      <c r="E179">
+        <v>0.4055</v>
+      </c>
+      <c r="F179" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="180" spans="1:6">
+      <c r="A180" t="s">
+        <v>21</v>
+      </c>
+      <c r="B180" t="s">
+        <v>41</v>
+      </c>
+      <c r="C180">
+        <v>1</v>
+      </c>
+      <c r="D180" t="s">
+        <v>170</v>
+      </c>
+      <c r="E180">
+        <v>0.0973</v>
+      </c>
+      <c r="F180" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="181" spans="1:6">
+      <c r="A181" t="s">
+        <v>21</v>
+      </c>
+      <c r="B181" t="s">
+        <v>41</v>
+      </c>
+      <c r="C181">
+        <v>2</v>
+      </c>
+      <c r="D181" t="s">
+        <v>171</v>
+      </c>
+      <c r="E181">
+        <v>0.1698</v>
+      </c>
+      <c r="F181" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="182" spans="1:6">
+      <c r="A182" t="s">
+        <v>21</v>
+      </c>
+      <c r="B182" t="s">
+        <v>41</v>
+      </c>
+      <c r="C182">
+        <v>3</v>
+      </c>
+      <c r="D182" t="s">
+        <v>172</v>
+      </c>
+      <c r="E182">
+        <v>0.1855</v>
+      </c>
+      <c r="F182" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="183" spans="1:6">
+      <c r="A183" t="s">
+        <v>21</v>
+      </c>
+      <c r="B183" t="s">
+        <v>41</v>
+      </c>
+      <c r="C183">
+        <v>4</v>
+      </c>
+      <c r="D183" t="s">
+        <v>173</v>
+      </c>
+      <c r="E183">
+        <v>0.2859</v>
+      </c>
+      <c r="F183" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="184" spans="1:6">
+      <c r="A184" t="s">
+        <v>21</v>
+      </c>
+      <c r="B184" t="s">
+        <v>41</v>
+      </c>
+      <c r="C184">
+        <v>5</v>
+      </c>
+      <c r="D184" t="s">
+        <v>174</v>
+      </c>
+      <c r="E184">
+        <v>0.3047</v>
+      </c>
+      <c r="F184" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="185" spans="1:6">
+      <c r="A185" t="s">
+        <v>21</v>
+      </c>
+      <c r="B185" t="s">
+        <v>41</v>
+      </c>
+      <c r="C185">
+        <v>6</v>
+      </c>
+      <c r="D185" t="s">
+        <v>175</v>
+      </c>
+      <c r="E185">
+        <v>0.1898</v>
+      </c>
+      <c r="F185" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="186" spans="1:6">
+      <c r="A186" t="s">
+        <v>21</v>
+      </c>
+      <c r="B186" t="s">
+        <v>41</v>
+      </c>
+      <c r="C186">
+        <v>7</v>
+      </c>
+      <c r="D186" t="s">
+        <v>176</v>
+      </c>
+      <c r="E186">
+        <v>0.1813</v>
+      </c>
+      <c r="F186" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="187" spans="1:6">
+      <c r="A187" t="s">
+        <v>21</v>
+      </c>
+      <c r="B187" t="s">
+        <v>41</v>
+      </c>
+      <c r="C187">
+        <v>8</v>
+      </c>
+      <c r="D187" t="s">
+        <v>177</v>
+      </c>
+      <c r="E187">
+        <v>0.082</v>
+      </c>
+      <c r="F187" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="188" spans="1:6">
+      <c r="A188" t="s">
+        <v>21</v>
+      </c>
+      <c r="B188" t="s">
+        <v>41</v>
+      </c>
+      <c r="C188">
+        <v>9</v>
+      </c>
+      <c r="D188" t="s">
+        <v>178</v>
+      </c>
+      <c r="E188">
+        <v>0.2175</v>
+      </c>
+      <c r="F188" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="189" spans="1:6">
+      <c r="A189" t="s">
+        <v>21</v>
+      </c>
+      <c r="B189" t="s">
+        <v>41</v>
+      </c>
+      <c r="C189">
+        <v>10</v>
+      </c>
+      <c r="D189" t="s">
+        <v>179</v>
+      </c>
+      <c r="E189">
+        <v>0.2137</v>
+      </c>
+      <c r="F189" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="190" spans="1:6">
+      <c r="A190" t="s">
+        <v>21</v>
+      </c>
+      <c r="B190" t="s">
+        <v>41</v>
+      </c>
+      <c r="C190">
+        <v>11</v>
+      </c>
+      <c r="D190" t="s">
+        <v>180</v>
+      </c>
+      <c r="E190">
+        <v>0.2007</v>
+      </c>
+      <c r="F190" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="191" spans="1:6">
+      <c r="A191" t="s">
+        <v>21</v>
+      </c>
+      <c r="B191" t="s">
+        <v>41</v>
+      </c>
+      <c r="C191">
+        <v>12</v>
+      </c>
+      <c r="D191" t="s">
+        <v>181</v>
+      </c>
+      <c r="E191">
+        <v>0.1036</v>
+      </c>
+      <c r="F191" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="192" spans="1:6">
+      <c r="A192" t="s">
+        <v>21</v>
+      </c>
+      <c r="B192" t="s">
+        <v>41</v>
+      </c>
+      <c r="C192">
+        <v>13</v>
+      </c>
+      <c r="D192" t="s">
+        <v>182</v>
+      </c>
+      <c r="E192">
+        <v>0.2143</v>
+      </c>
+      <c r="F192" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="193" spans="1:6">
+      <c r="A193" t="s">
+        <v>21</v>
+      </c>
+      <c r="B193" t="s">
+        <v>41</v>
+      </c>
+      <c r="C193">
+        <v>14</v>
+      </c>
+      <c r="D193" t="s">
+        <v>183</v>
+      </c>
+      <c r="E193">
+        <v>0.1146</v>
+      </c>
+      <c r="F193" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="194" spans="1:6">
+      <c r="A194" t="s">
+        <v>21</v>
+      </c>
+      <c r="B194" t="s">
+        <v>41</v>
+      </c>
+      <c r="C194">
+        <v>15</v>
+      </c>
+      <c r="D194" t="s">
+        <v>184</v>
+      </c>
+      <c r="E194">
+        <v>0.1555</v>
+      </c>
+      <c r="F194" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="195" spans="1:6">
+      <c r="A195" t="s">
+        <v>21</v>
+      </c>
+      <c r="B195" t="s">
+        <v>41</v>
+      </c>
+      <c r="C195">
+        <v>16</v>
+      </c>
+      <c r="D195" t="s">
+        <v>185</v>
+      </c>
+      <c r="E195">
+        <v>0.3266</v>
+      </c>
+      <c r="F195" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="196" spans="1:6">
+      <c r="A196" t="s">
+        <v>21</v>
+      </c>
+      <c r="B196" t="s">
+        <v>41</v>
+      </c>
+      <c r="C196">
+        <v>17</v>
+      </c>
+      <c r="D196" t="s">
+        <v>186</v>
+      </c>
+      <c r="E196">
+        <v>0.2117</v>
+      </c>
+      <c r="F196" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="197" spans="1:6">
+      <c r="A197" t="s">
+        <v>21</v>
+      </c>
+      <c r="B197" t="s">
+        <v>41</v>
+      </c>
+      <c r="C197">
+        <v>18</v>
+      </c>
+      <c r="D197" t="s">
+        <v>187</v>
+      </c>
+      <c r="E197">
+        <v>0.3606</v>
+      </c>
+      <c r="F197" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="198" spans="1:6">
+      <c r="A198" t="s">
+        <v>21</v>
+      </c>
+      <c r="B198" t="s">
+        <v>41</v>
+      </c>
+      <c r="C198">
+        <v>19</v>
+      </c>
+      <c r="D198" t="s">
+        <v>188</v>
+      </c>
+      <c r="E198">
+        <v>0.2731</v>
+      </c>
+      <c r="F198" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="199" spans="1:6">
+      <c r="A199" t="s">
+        <v>21</v>
+      </c>
+      <c r="B199" t="s">
+        <v>41</v>
+      </c>
+      <c r="C199">
+        <v>20</v>
+      </c>
+      <c r="D199" t="s">
+        <v>189</v>
+      </c>
+      <c r="E199">
+        <v>0.298</v>
+      </c>
+      <c r="F199" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="200" spans="1:6">
+      <c r="A200" t="s">
+        <v>21</v>
+      </c>
+      <c r="B200" t="s">
+        <v>41</v>
+      </c>
+      <c r="C200">
+        <v>21</v>
+      </c>
+      <c r="D200" t="s">
+        <v>190</v>
+      </c>
+      <c r="E200">
+        <v>0.2657</v>
+      </c>
+      <c r="F200" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="201" spans="1:6">
+      <c r="A201" t="s">
+        <v>21</v>
+      </c>
+      <c r="B201" t="s">
+        <v>41</v>
+      </c>
+      <c r="C201">
+        <v>22</v>
+      </c>
+      <c r="D201" t="s">
+        <v>191</v>
+      </c>
+      <c r="E201">
+        <v>0.2808</v>
+      </c>
+      <c r="F201" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="202" spans="1:6">
+      <c r="A202" t="s">
+        <v>21</v>
+      </c>
+      <c r="B202" t="s">
+        <v>41</v>
+      </c>
+      <c r="C202">
+        <v>23</v>
+      </c>
+      <c r="D202" t="s">
+        <v>192</v>
+      </c>
+      <c r="E202">
+        <v>0.2233</v>
+      </c>
+      <c r="F202" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="203" spans="1:6">
+      <c r="A203" t="s">
+        <v>21</v>
+      </c>
+      <c r="B203" t="s">
+        <v>41</v>
+      </c>
+      <c r="C203">
+        <v>24</v>
+      </c>
+      <c r="D203" t="s">
+        <v>193</v>
+      </c>
+      <c r="E203">
+        <v>0.1682</v>
+      </c>
+      <c r="F203" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="204" spans="1:6">
+      <c r="A204" t="s">
+        <v>22</v>
+      </c>
+      <c r="B204" t="s">
+        <v>42</v>
+      </c>
+      <c r="C204">
+        <v>1</v>
+      </c>
+      <c r="D204" t="s">
+        <v>194</v>
+      </c>
+      <c r="E204">
+        <v>0.18</v>
+      </c>
+      <c r="F204" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="205" spans="1:6">
+      <c r="A205" t="s">
+        <v>22</v>
+      </c>
+      <c r="B205" t="s">
+        <v>42</v>
+      </c>
+      <c r="C205">
+        <v>2</v>
+      </c>
+      <c r="D205" t="s">
+        <v>195</v>
+      </c>
+      <c r="E205">
+        <v>0.1933</v>
+      </c>
+      <c r="F205" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="206" spans="1:6">
+      <c r="A206" t="s">
+        <v>22</v>
+      </c>
+      <c r="B206" t="s">
+        <v>42</v>
+      </c>
+      <c r="C206">
+        <v>3</v>
+      </c>
+      <c r="D206" t="s">
+        <v>196</v>
+      </c>
+      <c r="E206">
+        <v>0.1658</v>
+      </c>
+      <c r="F206" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="207" spans="1:6">
+      <c r="A207" t="s">
+        <v>22</v>
+      </c>
+      <c r="B207" t="s">
+        <v>42</v>
+      </c>
+      <c r="C207">
+        <v>4</v>
+      </c>
+      <c r="D207" t="s">
+        <v>197</v>
+      </c>
+      <c r="E207">
+        <v>0.2125</v>
+      </c>
+      <c r="F207" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="208" spans="1:6">
+      <c r="A208" t="s">
+        <v>22</v>
+      </c>
+      <c r="B208" t="s">
+        <v>42</v>
+      </c>
+      <c r="C208">
+        <v>5</v>
+      </c>
+      <c r="D208" t="s">
+        <v>198</v>
+      </c>
+      <c r="E208">
+        <v>0.3514</v>
+      </c>
+      <c r="F208" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="209" spans="1:6">
+      <c r="A209" t="s">
+        <v>22</v>
+      </c>
+      <c r="B209" t="s">
+        <v>42</v>
+      </c>
+      <c r="C209">
+        <v>6</v>
+      </c>
+      <c r="D209" t="s">
+        <v>199</v>
+      </c>
+      <c r="E209">
+        <v>0.2825</v>
+      </c>
+      <c r="F209" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="210" spans="1:6">
+      <c r="A210" t="s">
+        <v>22</v>
+      </c>
+      <c r="B210" t="s">
+        <v>42</v>
+      </c>
+      <c r="C210">
+        <v>7</v>
+      </c>
+      <c r="D210" t="s">
+        <v>200</v>
+      </c>
+      <c r="E210">
+        <v>0.2293</v>
+      </c>
+      <c r="F210" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="211" spans="1:6">
+      <c r="A211" t="s">
+        <v>22</v>
+      </c>
+      <c r="B211" t="s">
+        <v>41</v>
+      </c>
+      <c r="C211" t="s">
+        <v>43</v>
+      </c>
+      <c r="D211" t="s">
+        <v>170</v>
+      </c>
+      <c r="E211">
+        <v>0.1449</v>
+      </c>
+      <c r="F211" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="212" spans="1:6">
+      <c r="A212" t="s">
+        <v>22</v>
+      </c>
+      <c r="B212" t="s">
+        <v>41</v>
+      </c>
+      <c r="C212" t="s">
+        <v>44</v>
+      </c>
+      <c r="D212" t="s">
+        <v>171</v>
+      </c>
+      <c r="E212">
+        <v>0.1865</v>
+      </c>
+      <c r="F212" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="213" spans="1:6">
+      <c r="A213" t="s">
+        <v>22</v>
+      </c>
+      <c r="B213" t="s">
+        <v>41</v>
+      </c>
+      <c r="C213" t="s">
+        <v>45</v>
+      </c>
+      <c r="D213" t="s">
+        <v>172</v>
+      </c>
+      <c r="E213">
+        <v>0.2748</v>
+      </c>
+      <c r="F213" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="214" spans="1:6">
+      <c r="A214" t="s">
+        <v>22</v>
+      </c>
+      <c r="B214" t="s">
+        <v>41</v>
+      </c>
+      <c r="C214" t="s">
+        <v>46</v>
+      </c>
+      <c r="D214" t="s">
+        <v>173</v>
+      </c>
+      <c r="E214">
+        <v>0.3114</v>
+      </c>
+      <c r="F214" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="215" spans="1:6">
+      <c r="A215" t="s">
+        <v>22</v>
+      </c>
+      <c r="B215" t="s">
+        <v>41</v>
+      </c>
+      <c r="C215" t="s">
+        <v>47</v>
+      </c>
+      <c r="D215" t="s">
+        <v>174</v>
+      </c>
+      <c r="E215">
+        <v>0.3704</v>
+      </c>
+      <c r="F215" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="216" spans="1:6">
+      <c r="A216" t="s">
+        <v>22</v>
+      </c>
+      <c r="B216" t="s">
+        <v>41</v>
+      </c>
+      <c r="C216" t="s">
+        <v>48</v>
+      </c>
+      <c r="D216" t="s">
+        <v>175</v>
+      </c>
+      <c r="E216">
+        <v>0.2685</v>
+      </c>
+      <c r="F216" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="217" spans="1:6">
+      <c r="A217" t="s">
+        <v>22</v>
+      </c>
+      <c r="B217" t="s">
+        <v>41</v>
+      </c>
+      <c r="C217" t="s">
+        <v>49</v>
+      </c>
+      <c r="D217" t="s">
+        <v>176</v>
+      </c>
+      <c r="E217">
+        <v>0.1876</v>
+      </c>
+      <c r="F217" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="218" spans="1:6">
+      <c r="A218" t="s">
+        <v>22</v>
+      </c>
+      <c r="B218" t="s">
+        <v>41</v>
+      </c>
+      <c r="C218" t="s">
+        <v>50</v>
+      </c>
+      <c r="D218" t="s">
+        <v>177</v>
+      </c>
+      <c r="E218">
+        <v>0.1371</v>
+      </c>
+      <c r="F218" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="219" spans="1:6">
+      <c r="A219" t="s">
+        <v>22</v>
+      </c>
+      <c r="B219" t="s">
+        <v>41</v>
+      </c>
+      <c r="C219" t="s">
+        <v>51</v>
+      </c>
+      <c r="D219" t="s">
+        <v>178</v>
+      </c>
+      <c r="E219">
+        <v>0.2504</v>
+      </c>
+      <c r="F219" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="220" spans="1:6">
+      <c r="A220" t="s">
+        <v>22</v>
+      </c>
+      <c r="B220" t="s">
+        <v>41</v>
+      </c>
+      <c r="C220" t="s">
+        <v>52</v>
+      </c>
+      <c r="D220" t="s">
+        <v>179</v>
+      </c>
+      <c r="E220">
+        <v>0.2874</v>
+      </c>
+      <c r="F220" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="221" spans="1:6">
+      <c r="A221" t="s">
+        <v>22</v>
+      </c>
+      <c r="B221" t="s">
+        <v>41</v>
+      </c>
+      <c r="C221" t="s">
+        <v>53</v>
+      </c>
+      <c r="D221" t="s">
+        <v>180</v>
+      </c>
+      <c r="E221">
+        <v>0.2726</v>
+      </c>
+      <c r="F221" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="222" spans="1:6">
+      <c r="A222" t="s">
+        <v>22</v>
+      </c>
+      <c r="B222" t="s">
+        <v>41</v>
+      </c>
+      <c r="C222" t="s">
+        <v>54</v>
+      </c>
+      <c r="D222" t="s">
+        <v>181</v>
+      </c>
+      <c r="E222">
+        <v>0.1568</v>
+      </c>
+      <c r="F222" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="223" spans="1:6">
+      <c r="A223" t="s">
+        <v>22</v>
+      </c>
+      <c r="B223" t="s">
+        <v>41</v>
+      </c>
+      <c r="C223" t="s">
+        <v>55</v>
+      </c>
+      <c r="D223" t="s">
+        <v>182</v>
+      </c>
+      <c r="E223">
+        <v>0.2373</v>
+      </c>
+      <c r="F223" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="224" spans="1:6">
+      <c r="A224" t="s">
+        <v>22</v>
+      </c>
+      <c r="B224" t="s">
+        <v>41</v>
+      </c>
+      <c r="C224" t="s">
+        <v>56</v>
+      </c>
+      <c r="D224" t="s">
+        <v>183</v>
+      </c>
+      <c r="E224">
+        <v>0.2109</v>
+      </c>
+      <c r="F224" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="225" spans="1:6">
+      <c r="A225" t="s">
+        <v>22</v>
+      </c>
+      <c r="B225" t="s">
+        <v>41</v>
+      </c>
+      <c r="C225" t="s">
+        <v>57</v>
+      </c>
+      <c r="D225" t="s">
+        <v>184</v>
+      </c>
+      <c r="E225">
+        <v>0.2147</v>
+      </c>
+      <c r="F225" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="226" spans="1:6">
+      <c r="A226" t="s">
+        <v>22</v>
+      </c>
+      <c r="B226" t="s">
+        <v>41</v>
+      </c>
+      <c r="C226" t="s">
+        <v>58</v>
+      </c>
+      <c r="D226" t="s">
+        <v>185</v>
+      </c>
+      <c r="E226">
+        <v>0.3517</v>
+      </c>
+      <c r="F226" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="227" spans="1:6">
+      <c r="A227" t="s">
+        <v>22</v>
+      </c>
+      <c r="B227" t="s">
+        <v>41</v>
+      </c>
+      <c r="C227" t="s">
+        <v>59</v>
+      </c>
+      <c r="D227" t="s">
+        <v>186</v>
+      </c>
+      <c r="E227">
+        <v>0.2691</v>
+      </c>
+      <c r="F227" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="228" spans="1:6">
+      <c r="A228" t="s">
+        <v>22</v>
+      </c>
+      <c r="B228" t="s">
+        <v>41</v>
+      </c>
+      <c r="C228" t="s">
+        <v>60</v>
+      </c>
+      <c r="D228" t="s">
+        <v>187</v>
+      </c>
+      <c r="E228">
+        <v>0.4198</v>
+      </c>
+      <c r="F228" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="229" spans="1:6">
+      <c r="A229" t="s">
+        <v>22</v>
+      </c>
+      <c r="B229" t="s">
+        <v>41</v>
+      </c>
+      <c r="C229" t="s">
+        <v>61</v>
+      </c>
+      <c r="D229" t="s">
+        <v>188</v>
+      </c>
+      <c r="E229">
+        <v>0.3182</v>
+      </c>
+      <c r="F229" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="230" spans="1:6">
+      <c r="A230" t="s">
+        <v>22</v>
+      </c>
+      <c r="B230" t="s">
+        <v>41</v>
+      </c>
+      <c r="C230" t="s">
+        <v>62</v>
+      </c>
+      <c r="D230" t="s">
+        <v>189</v>
+      </c>
+      <c r="E230">
+        <v>0.4125</v>
+      </c>
+      <c r="F230" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="231" spans="1:6">
+      <c r="A231" t="s">
+        <v>22</v>
+      </c>
+      <c r="B231" t="s">
+        <v>41</v>
+      </c>
+      <c r="C231" t="s">
+        <v>63</v>
+      </c>
+      <c r="D231" t="s">
+        <v>190</v>
+      </c>
+      <c r="E231">
+        <v>0.3677</v>
+      </c>
+      <c r="F231" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="232" spans="1:6">
+      <c r="A232" t="s">
+        <v>22</v>
+      </c>
+      <c r="B232" t="s">
+        <v>41</v>
+      </c>
+      <c r="C232" t="s">
+        <v>64</v>
+      </c>
+      <c r="D232" t="s">
+        <v>191</v>
+      </c>
+      <c r="E232">
+        <v>0.3396</v>
+      </c>
+      <c r="F232" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="233" spans="1:6">
+      <c r="A233" t="s">
+        <v>22</v>
+      </c>
+      <c r="B233" t="s">
+        <v>41</v>
+      </c>
+      <c r="C233" t="s">
+        <v>65</v>
+      </c>
+      <c r="D233" t="s">
+        <v>192</v>
+      </c>
+      <c r="E233">
+        <v>0.2825</v>
+      </c>
+      <c r="F233" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="234" spans="1:6">
+      <c r="A234" t="s">
+        <v>22</v>
+      </c>
+      <c r="B234" t="s">
+        <v>41</v>
+      </c>
+      <c r="C234" t="s">
+        <v>66</v>
+      </c>
+      <c r="D234" t="s">
+        <v>193</v>
+      </c>
+      <c r="E234">
+        <v>0.2293</v>
+      </c>
+      <c r="F234" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>